<commit_message>
replaced another winner with suspicious journal entry
</commit_message>
<xml_diff>
--- a/outputs/final_consolation_200_excluding_selected.xlsx
+++ b/outputs/final_consolation_200_excluding_selected.xlsx
@@ -23093,12 +23093,12 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>Ravi Kumar</t>
+          <t>Saiful Haizam</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>1558303682</t>
+          <t>537089163</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23121,51 +23121,51 @@
       </c>
       <c r="I199" t="inlineStr">
         <is>
-          <t>2026-04-15 21:55:40 GMT+8</t>
+          <t>2026-03-16 23:30:39 GMT+8</t>
         </is>
       </c>
       <c r="J199" t="inlineStr">
         <is>
-          <t>2026-04-15 21:57:12 GMT+8</t>
+          <t>2026-03-16 23:34:04 GMT+8</t>
         </is>
       </c>
       <c r="K199" t="inlineStr">
         <is>
-          <t>2026-04-15 21:55:20 GMT+8</t>
+          <t>2026-03-16 23:24:24 GMT+8</t>
         </is>
       </c>
       <c r="L199" t="inlineStr">
         <is>
-          <t>2026-04-15 21:54:41 GMT+8</t>
+          <t>2026-02-20 22:23:49 GMT+8</t>
         </is>
       </c>
       <c r="M199" t="n">
-        <v>35766</v>
+        <v>15579</v>
       </c>
       <c r="N199" t="inlineStr">
         <is>
-          <t>2026-04-15 21:57:12 GMT+8</t>
+          <t>2026-03-16 23:30:39 GMT+8</t>
         </is>
       </c>
       <c r="O199" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/share/p/1BMM3FeM3B/</t>
+          <t>Saya berkongsi rezeki dengan membeli Tropicana Twister dan kemudian diagih-agihkan kepada jiran tetangga</t>
         </is>
       </c>
       <c r="P199" t="n">
-        <v>44</v>
+        <v>104</v>
       </c>
       <c r="Q199" t="n">
-        <v>1.1</v>
+        <v>-2.4</v>
       </c>
       <c r="R199" t="n">
-        <v>1.1</v>
+        <v>2.6</v>
       </c>
       <c r="S199" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="T199" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="U199" t="n">
         <v>0</v>
@@ -23177,13 +23177,13 @@
         <v>0</v>
       </c>
       <c r="X199" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="Y199" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Z199" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA199" t="n">
         <v>0</v>
@@ -23208,12 +23208,12 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>Saiful Haizam</t>
+          <t>Salmah Jaafar</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>537089163</t>
+          <t>26750312877989179</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23236,48 +23236,48 @@
       </c>
       <c r="I200" t="inlineStr">
         <is>
-          <t>2026-03-16 23:30:39 GMT+8</t>
+          <t>2026-04-12 09:42:11 GMT+8</t>
         </is>
       </c>
       <c r="J200" t="inlineStr">
         <is>
-          <t>2026-03-16 23:34:04 GMT+8</t>
+          <t>2026-04-12 09:43:52 GMT+8</t>
         </is>
       </c>
       <c r="K200" t="inlineStr">
         <is>
-          <t>2026-03-16 23:24:24 GMT+8</t>
+          <t>2026-04-12 09:40:28 GMT+8</t>
         </is>
       </c>
       <c r="L200" t="inlineStr">
         <is>
-          <t>2026-02-20 22:23:49 GMT+8</t>
+          <t>2026-04-12 09:40:28 GMT+8</t>
         </is>
       </c>
       <c r="M200" t="n">
-        <v>15579</v>
+        <v>33096</v>
       </c>
       <c r="N200" t="inlineStr">
         <is>
-          <t>2026-03-16 23:30:39 GMT+8</t>
+          <t>2026-04-12 09:43:52 GMT+8</t>
         </is>
       </c>
       <c r="O200" t="inlineStr">
         <is>
-          <t>Saya berkongsi rezeki dengan membeli Tropicana Twister dan kemudian diagih-agihkan kepada jiran tetangga</t>
+          <t>Saya bantu orang menunjukan jalan.</t>
         </is>
       </c>
       <c r="P200" t="n">
-        <v>104</v>
+        <v>34</v>
       </c>
       <c r="Q200" t="n">
-        <v>-2.4</v>
+        <v>10.85</v>
       </c>
       <c r="R200" t="n">
-        <v>2.6</v>
+        <v>0.85</v>
       </c>
       <c r="S200" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="T200" t="n">
         <v>5</v>
@@ -23292,10 +23292,10 @@
         <v>0</v>
       </c>
       <c r="X200" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="Y200" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Z200" t="n">
         <v>1</v>
@@ -23323,12 +23323,12 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>Salmah Jaafar</t>
+          <t>Sariffudin Fiza</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>26750312877989179</t>
+          <t>25640455475627828</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23351,48 +23351,48 @@
       </c>
       <c r="I201" t="inlineStr">
         <is>
-          <t>2026-04-12 09:42:11 GMT+8</t>
+          <t>2026-04-17 15:40:28 GMT+8</t>
         </is>
       </c>
       <c r="J201" t="inlineStr">
         <is>
-          <t>2026-04-12 09:43:52 GMT+8</t>
+          <t>2026-04-17 16:13:56 GMT+8</t>
         </is>
       </c>
       <c r="K201" t="inlineStr">
         <is>
-          <t>2026-04-12 09:40:28 GMT+8</t>
+          <t>2026-04-17 16:12:47 GMT+8</t>
         </is>
       </c>
       <c r="L201" t="inlineStr">
         <is>
-          <t>2026-04-12 09:40:28 GMT+8</t>
+          <t>2026-04-17 15:39:37 GMT+8</t>
         </is>
       </c>
       <c r="M201" t="n">
-        <v>33096</v>
+        <v>36502</v>
       </c>
       <c r="N201" t="inlineStr">
         <is>
-          <t>2026-04-12 09:43:52 GMT+8</t>
+          <t>2026-04-17 15:40:28 GMT+8</t>
         </is>
       </c>
       <c r="O201" t="inlineStr">
         <is>
-          <t>Saya bantu orang menunjukan jalan.</t>
+          <t>saya sayang family saya</t>
         </is>
       </c>
       <c r="P201" t="n">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="Q201" t="n">
-        <v>10.85</v>
+        <v>-9.43</v>
       </c>
       <c r="R201" t="n">
-        <v>0.85</v>
+        <v>0.575</v>
       </c>
       <c r="S201" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="T201" t="n">
         <v>5</v>
@@ -23404,13 +23404,13 @@
         <v>0</v>
       </c>
       <c r="W201" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="X201" t="n">
         <v>0</v>
       </c>
       <c r="Y201" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Z201" t="n">
         <v>1</v>
@@ -23422,7 +23422,7 @@
         <v>0</v>
       </c>
       <c r="AC201" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AD201" t="inlineStr">
         <is>

</xml_diff>